<commit_message>
Updated owner WhatsApp number in confirmation modal to 917984183225
</commit_message>
<xml_diff>
--- a/data/b2b_bookings.xlsx
+++ b/data/b2b_bookings.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="69">
   <si>
     <t>Booking ID</t>
   </si>
@@ -43,15 +43,84 @@
     <t>Created At (Timestamp)</t>
   </si>
   <si>
+    <t>B2B-5148</t>
+  </si>
+  <si>
+    <t>Priya Sharma</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>Luxury Glow Facial &amp; Cleanups</t>
+  </si>
+  <si>
+    <t>₹0</t>
+  </si>
+  <si>
+    <t>2025-03-25</t>
+  </si>
+  <si>
+    <t>11:00 AM (Morning)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>30/9/2026, 11:35:36 am</t>
+  </si>
+  <si>
+    <t>B2B-4471</t>
+  </si>
+  <si>
+    <t>Barath</t>
+  </si>
+  <si>
+    <t>8189909510</t>
+  </si>
+  <si>
+    <t>₹1999</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>30/9/2026, 11:12:53 am</t>
+  </si>
+  <si>
+    <t>B2B-6589</t>
+  </si>
+  <si>
+    <t>7904183225</t>
+  </si>
+  <si>
+    <t>Hair Styling &amp; Spa</t>
+  </si>
+  <si>
+    <t>₹1499</t>
+  </si>
+  <si>
+    <t>01:30 PM (Afternoon)</t>
+  </si>
+  <si>
+    <t>30/9/2026, 11:06:55 am</t>
+  </si>
+  <si>
+    <t>B2B-5420</t>
+  </si>
+  <si>
+    <t>30/9/2026, 11:04:32 am</t>
+  </si>
+  <si>
     <t>B2B-1305</t>
   </si>
   <si>
     <t>Mahendran</t>
   </si>
   <si>
-    <t>7904183225</t>
-  </si>
-  <si>
     <t>Bridal &amp; Event Makeover Packages</t>
   </si>
   <si>
@@ -64,9 +133,6 @@
     <t>05:30 PM (Evening)</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
     <t>Confirmed</t>
   </si>
   <si>
@@ -76,15 +142,9 @@
     <t>B2B-6893</t>
   </si>
   <si>
-    <t>Barath</t>
-  </si>
-  <si>
     <t>2025-03-20</t>
   </si>
   <si>
-    <t>01:30 PM (Afternoon)</t>
-  </si>
-  <si>
     <t>Bridal makeover for reception</t>
   </si>
   <si>
@@ -94,18 +154,9 @@
     <t>B2B-8420</t>
   </si>
   <si>
-    <t>Luxury Glow Facial &amp; Cleanups</t>
-  </si>
-  <si>
-    <t>₹1999</t>
-  </si>
-  <si>
     <t>2025-03-12</t>
   </si>
   <si>
-    <t>11:00 AM (Morning)</t>
-  </si>
-  <si>
     <t>B2B Test</t>
   </si>
   <si>
@@ -124,12 +175,6 @@
     <t>B2B-6574</t>
   </si>
   <si>
-    <t>Hair Styling &amp; Spa</t>
-  </si>
-  <si>
-    <t>₹1499</t>
-  </si>
-  <si>
     <t>2026-09-27</t>
   </si>
   <si>
@@ -140,12 +185,6 @@
   </si>
   <si>
     <t>B2B-8901</t>
-  </si>
-  <si>
-    <t>Priya Sharma</t>
-  </si>
-  <si>
-    <t>9876543210</t>
   </si>
   <si>
     <t>2025-03-05</t>
@@ -201,11 +240,11 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF008000"/>
+      <color rgb="FFD4AF37"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFD4AF37"/>
+      <color rgb="FF008000"/>
     </font>
     <font>
       <b/>
@@ -593,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -680,22 +719,22 @@
         <v>21</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>18</v>
@@ -712,83 +751,83 @@
         <v>21</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>30</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>30</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>18</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>17</v>
@@ -805,63 +844,191 @@
         <v>42</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>45</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>30</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>40</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="I9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="2" t="s">
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="B10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="G10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>55</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replaced owner mobile number with 7904183225 across backend and frontend
</commit_message>
<xml_diff>
--- a/data/b2b_bookings.xlsx
+++ b/data/b2b_bookings.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="75">
   <si>
     <t>Booking ID</t>
   </si>
@@ -43,6 +43,36 @@
     <t>Created At (Timestamp)</t>
   </si>
   <si>
+    <t>B2B-9001</t>
+  </si>
+  <si>
+    <t>jeyandhan</t>
+  </si>
+  <si>
+    <t>9566221144</t>
+  </si>
+  <si>
+    <t>Threading &amp; Skin Care</t>
+  </si>
+  <si>
+    <t>₹499</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>11:00 AM (Morning)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>30/9/2026, 11:49:12 am</t>
+  </si>
+  <si>
     <t>B2B-5148</t>
   </si>
   <si>
@@ -61,15 +91,6 @@
     <t>2025-03-25</t>
   </si>
   <si>
-    <t>11:00 AM (Morning)</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Pending</t>
-  </si>
-  <si>
     <t>30/9/2026, 11:35:36 am</t>
   </si>
   <si>
@@ -83,9 +104,6 @@
   </si>
   <si>
     <t>₹1999</t>
-  </si>
-  <si>
-    <t>2026-10-01</t>
   </si>
   <si>
     <t>30/9/2026, 11:12:53 am</t>
@@ -632,7 +650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -722,13 +740,13 @@
         <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>16</v>
@@ -740,30 +758,30 @@
         <v>18</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>17</v>
@@ -780,22 +798,22 @@
         <v>32</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>17</v>
@@ -804,231 +822,263 @@
         <v>18</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="F6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>40</v>
+      <c r="I6" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="J8" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="G10" s="2" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>46</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>64</v>
       </c>
       <c r="G12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="I12" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I12" s="5" t="s">
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>68</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added localtunnel startup and dedicated POST /api/book-appointment route
</commit_message>
<xml_diff>
--- a/data/b2b_bookings.xlsx
+++ b/data/b2b_bookings.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="80">
   <si>
     <t>Booking ID</t>
   </si>
@@ -43,15 +43,39 @@
     <t>Created At (Timestamp)</t>
   </si>
   <si>
+    <t>B2B-7564</t>
+  </si>
+  <si>
+    <t>jeyandhan</t>
+  </si>
+  <si>
+    <t>9566221144</t>
+  </si>
+  <si>
+    <t>Manicure &amp; Pedicure Spa</t>
+  </si>
+  <si>
+    <t>₹999</t>
+  </si>
+  <si>
+    <t>2026-10-03</t>
+  </si>
+  <si>
+    <t>01:30 PM (Afternoon)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Confirmed</t>
+  </si>
+  <si>
+    <t>30/9/2026, 11:55:11 am</t>
+  </si>
+  <si>
     <t>B2B-9001</t>
   </si>
   <si>
-    <t>jeyandhan</t>
-  </si>
-  <si>
-    <t>9566221144</t>
-  </si>
-  <si>
     <t>Threading &amp; Skin Care</t>
   </si>
   <si>
@@ -64,9 +88,6 @@
     <t>11:00 AM (Morning)</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
     <t>Pending</t>
   </si>
   <si>
@@ -121,9 +142,6 @@
     <t>₹1499</t>
   </si>
   <si>
-    <t>01:30 PM (Afternoon)</t>
-  </si>
-  <si>
     <t>30/9/2026, 11:06:55 am</t>
   </si>
   <si>
@@ -149,9 +167,6 @@
   </si>
   <si>
     <t>05:30 PM (Evening)</t>
-  </si>
-  <si>
-    <t>Confirmed</t>
   </si>
   <si>
     <t>27/9/2026, 12:47:08 pm</t>
@@ -258,11 +273,11 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFD4AF37"/>
+      <color rgb="FF008000"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF008000"/>
+      <color rgb="FFD4AF37"/>
     </font>
     <font>
       <b/>
@@ -650,7 +665,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -734,28 +749,28 @@
         <v>20</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>18</v>
+      <c r="I3" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>26</v>
@@ -772,313 +787,345 @@
         <v>29</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>18</v>
+      <c r="I4" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>18</v>
+      <c r="I5" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="3" t="s">
-        <v>18</v>
+      <c r="I6" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="F7" s="2" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="E8" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>46</v>
+        <v>17</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>46</v>
+        <v>55</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>46</v>
+        <v>59</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>61</v>
+        <v>18</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>61</v>
+        <v>17</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>66</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="I13" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="H13" s="2" t="s">
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="B14" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>74</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Integrated MongoDB Mongoose cloud database connector with dual JSON and Excel sync
</commit_message>
<xml_diff>
--- a/data/b2b_bookings.xlsx
+++ b/data/b2b_bookings.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="84">
   <si>
     <t>Booking ID</t>
   </si>
@@ -43,6 +43,36 @@
     <t>Created At (Timestamp)</t>
   </si>
   <si>
+    <t>B2B-5564</t>
+  </si>
+  <si>
+    <t>jeevi</t>
+  </si>
+  <si>
+    <t>7894561234</t>
+  </si>
+  <si>
+    <t>Hair Styling &amp; Spa</t>
+  </si>
+  <si>
+    <t>₹1499</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>11:00 AM (Morning)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Confirmed</t>
+  </si>
+  <si>
+    <t>1/10/2026, 11:55:50 am</t>
+  </si>
+  <si>
     <t>B2B-7564</t>
   </si>
   <si>
@@ -64,12 +94,6 @@
     <t>01:30 PM (Afternoon)</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Confirmed</t>
-  </si>
-  <si>
     <t>30/9/2026, 11:55:11 am</t>
   </si>
   <si>
@@ -82,12 +106,6 @@
     <t>₹499</t>
   </si>
   <si>
-    <t>2026-10-01</t>
-  </si>
-  <si>
-    <t>11:00 AM (Morning)</t>
-  </si>
-  <si>
     <t>Pending</t>
   </si>
   <si>
@@ -134,12 +152,6 @@
   </si>
   <si>
     <t>7904183225</t>
-  </si>
-  <si>
-    <t>Hair Styling &amp; Spa</t>
-  </si>
-  <si>
-    <t>₹1499</t>
   </si>
   <si>
     <t>30/9/2026, 11:06:55 am</t>
@@ -665,7 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -749,115 +761,115 @@
         <v>20</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>25</v>
+      <c r="I3" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>37</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>16</v>
@@ -866,100 +878,100 @@
         <v>17</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>41</v>
+        <v>13</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="3" t="s">
-        <v>18</v>
+      <c r="I8" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>49</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>54</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>18</v>
@@ -973,22 +985,22 @@
         <v>57</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>58</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>59</v>
@@ -1005,60 +1017,60 @@
         <v>61</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>18</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I12" s="4" t="s">
         <v>66</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>67</v>
@@ -1069,28 +1081,28 @@
         <v>68</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>69</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>71</v>
@@ -1101,31 +1113,63 @@
         <v>72</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="G14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="I14" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="G14" s="2" t="s">
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="C15" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>79</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed customerName overwrite bug and added SSE deduplication in Admin dashboard
</commit_message>
<xml_diff>
--- a/data/b2b_bookings.xlsx
+++ b/data/b2b_bookings.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="97">
   <si>
     <t>Booking ID</t>
   </si>
@@ -43,6 +43,63 @@
     <t>Created At (Timestamp)</t>
   </si>
   <si>
+    <t>B2B-7652</t>
+  </si>
+  <si>
+    <t>Guest Customer</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Beauty Treatment</t>
+  </si>
+  <si>
+    <t>₹0</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>11:00 AM (Morning)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Confirmed</t>
+  </si>
+  <si>
+    <t>1/10/2026, 6:21:22 pm</t>
+  </si>
+  <si>
+    <t>B2B-7007</t>
+  </si>
+  <si>
+    <t>1/10/2026, 6:20:47 pm</t>
+  </si>
+  <si>
+    <t>B2B-5589</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>1/10/2026, 6:20:31 pm</t>
+  </si>
+  <si>
+    <t>B2B-6378</t>
+  </si>
+  <si>
+    <t>1/10/2026, 6:16:45 pm</t>
+  </si>
+  <si>
+    <t>B2B-9161</t>
+  </si>
+  <si>
+    <t>1/10/2026, 6:16:35 pm</t>
+  </si>
+  <si>
     <t>B2B-5564</t>
   </si>
   <si>
@@ -58,18 +115,6 @@
     <t>₹1499</t>
   </si>
   <si>
-    <t>2026-10-01</t>
-  </si>
-  <si>
-    <t>11:00 AM (Morning)</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Confirmed</t>
-  </si>
-  <si>
     <t>1/10/2026, 11:55:50 am</t>
   </si>
   <si>
@@ -106,9 +151,6 @@
     <t>₹499</t>
   </si>
   <si>
-    <t>Pending</t>
-  </si>
-  <si>
     <t>30/9/2026, 11:49:12 am</t>
   </si>
   <si>
@@ -122,9 +164,6 @@
   </si>
   <si>
     <t>Luxury Glow Facial &amp; Cleanups</t>
-  </si>
-  <si>
-    <t>₹0</t>
   </si>
   <si>
     <t>2025-03-25</t>
@@ -677,7 +716,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -761,22 +800,22 @@
         <v>20</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>17</v>
@@ -785,24 +824,24 @@
         <v>18</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>15</v>
@@ -814,30 +853,30 @@
         <v>17</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>16</v>
@@ -845,28 +884,28 @@
       <c r="H5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>31</v>
+      <c r="I5" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>15</v>
@@ -877,299 +916,459 @@
       <c r="H6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>31</v>
+      <c r="I6" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="4" t="s">
-        <v>31</v>
+      <c r="I7" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="4" t="s">
-        <v>31</v>
+      <c r="I8" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="3" t="s">
-        <v>18</v>
+      <c r="I9" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="H12" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>70</v>
+        <v>17</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="I16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C15" s="2" t="s">
+    </row>
+    <row r="17" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F15" s="2" t="s">
+      <c r="B17" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="I17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="H15" s="2" t="s">
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="B18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="G18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="4" t="s">
         <v>83</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Unified GET /api/appointments dataset merging and added 5s auto polling on Admin dashboard
</commit_message>
<xml_diff>
--- a/data/b2b_bookings.xlsx
+++ b/data/b2b_bookings.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="70">
   <si>
     <t>Booking ID</t>
   </si>
@@ -46,16 +46,16 @@
     <t>B2B-7652</t>
   </si>
   <si>
-    <t>Guest Customer</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Beauty Treatment</t>
-  </si>
-  <si>
-    <t>₹0</t>
+    <t>Prem</t>
+  </si>
+  <si>
+    <t>7458693210</t>
+  </si>
+  <si>
+    <t>Luxury Glow Facial &amp; Cleanups</t>
+  </si>
+  <si>
+    <t>₹1999</t>
   </si>
   <si>
     <t>2026-10-01</t>
@@ -73,31 +73,58 @@
     <t>1/10/2026, 6:21:22 pm</t>
   </si>
   <si>
-    <t>B2B-7007</t>
-  </si>
-  <si>
-    <t>1/10/2026, 6:20:47 pm</t>
-  </si>
-  <si>
-    <t>B2B-5589</t>
+    <t>B2B-6378</t>
+  </si>
+  <si>
+    <t>9632581470</t>
+  </si>
+  <si>
+    <t>Bridal &amp; Event Makeover Packages</t>
+  </si>
+  <si>
+    <t>₹7999</t>
+  </si>
+  <si>
+    <t>1/10/2026, 6:16:45 pm</t>
+  </si>
+  <si>
+    <t>B2B-9161</t>
+  </si>
+  <si>
+    <t>Ammu</t>
+  </si>
+  <si>
+    <t>7904183226</t>
+  </si>
+  <si>
+    <t>2026-10-02</t>
+  </si>
+  <si>
+    <t>05:30 PM (Evening)</t>
+  </si>
+  <si>
+    <t>1/10/2026, 6:16:35 pm</t>
+  </si>
+  <si>
+    <t>B2B-5019</t>
+  </si>
+  <si>
+    <t>Jithin</t>
+  </si>
+  <si>
+    <t>9865321478</t>
+  </si>
+  <si>
+    <t>Hair Styling &amp; Spa</t>
+  </si>
+  <si>
+    <t>₹1499</t>
   </si>
   <si>
     <t>Pending</t>
   </si>
   <si>
-    <t>1/10/2026, 6:20:31 pm</t>
-  </si>
-  <si>
-    <t>B2B-6378</t>
-  </si>
-  <si>
-    <t>1/10/2026, 6:16:45 pm</t>
-  </si>
-  <si>
-    <t>B2B-9161</t>
-  </si>
-  <si>
-    <t>1/10/2026, 6:16:35 pm</t>
+    <t>1/10/2026, 1:42:00 pm</t>
   </si>
   <si>
     <t>B2B-5564</t>
@@ -109,12 +136,6 @@
     <t>7894561234</t>
   </si>
   <si>
-    <t>Hair Styling &amp; Spa</t>
-  </si>
-  <si>
-    <t>₹1499</t>
-  </si>
-  <si>
     <t>1/10/2026, 11:55:50 am</t>
   </si>
   <si>
@@ -163,9 +184,6 @@
     <t>9876543210</t>
   </si>
   <si>
-    <t>Luxury Glow Facial &amp; Cleanups</t>
-  </si>
-  <si>
     <t>2025-03-25</t>
   </si>
   <si>
@@ -181,9 +199,6 @@
     <t>8189909510</t>
   </si>
   <si>
-    <t>₹1999</t>
-  </si>
-  <si>
     <t>30/9/2026, 11:12:53 am</t>
   </si>
   <si>
@@ -196,119 +211,23 @@
     <t>30/9/2026, 11:06:55 am</t>
   </si>
   <si>
-    <t>B2B-5420</t>
-  </si>
-  <si>
-    <t>30/9/2026, 11:04:32 am</t>
-  </si>
-  <si>
     <t>B2B-1305</t>
   </si>
   <si>
     <t>Mahendran</t>
   </si>
   <si>
-    <t>Bridal &amp; Event Makeover Packages</t>
-  </si>
-  <si>
-    <t>₹7999</t>
-  </si>
-  <si>
     <t>2026-09-28</t>
   </si>
   <si>
-    <t>05:30 PM (Evening)</t>
-  </si>
-  <si>
     <t>27/9/2026, 12:47:08 pm</t>
-  </si>
-  <si>
-    <t>B2B-6893</t>
-  </si>
-  <si>
-    <t>2025-03-20</t>
-  </si>
-  <si>
-    <t>Bridal makeover for reception</t>
-  </si>
-  <si>
-    <t>27/9/2026, 12:23:57 pm</t>
-  </si>
-  <si>
-    <t>B2B-8420</t>
-  </si>
-  <si>
-    <t>2025-03-12</t>
-  </si>
-  <si>
-    <t>B2B Test</t>
-  </si>
-  <si>
-    <t>27/9/2026, 12:13:32 pm</t>
-  </si>
-  <si>
-    <t>AURA-4576</t>
-  </si>
-  <si>
-    <t>Replaced brand name to B2B</t>
-  </si>
-  <si>
-    <t>27/9/2026, 12:11:05 pm</t>
-  </si>
-  <si>
-    <t>B2B-6574</t>
-  </si>
-  <si>
-    <t>2026-09-27</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>27/9/2026, 11:57:00 am</t>
-  </si>
-  <si>
-    <t>B2B-8901</t>
-  </si>
-  <si>
-    <t>2025-03-05</t>
-  </si>
-  <si>
-    <t>Prefers gentle pressure and organic skin products.</t>
-  </si>
-  <si>
-    <t>1/3/2025, 3:45:00 pm</t>
-  </si>
-  <si>
-    <t>B2B-8902</t>
-  </si>
-  <si>
-    <t>Ananya Roy</t>
-  </si>
-  <si>
-    <t>9123456789</t>
-  </si>
-  <si>
-    <t>2025-03-06</t>
-  </si>
-  <si>
-    <t>02:30 PM (Afternoon)</t>
-  </si>
-  <si>
-    <t>Reception makeup trial session.</t>
-  </si>
-  <si>
-    <t>Cancelled</t>
-  </si>
-  <si>
-    <t>1/3/2025, 5:15:00 pm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -329,10 +248,6 @@
     <font>
       <b/>
       <color rgb="FFD4AF37"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFCC0000"/>
     </font>
   </fonts>
   <fills count="3">
@@ -360,7 +275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -372,9 +287,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -716,7 +628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -803,13 +715,13 @@
         <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>15</v>
@@ -824,56 +736,56 @@
         <v>18</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="4" t="s">
-        <v>23</v>
+      <c r="I4" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>15</v>
@@ -884,28 +796,28 @@
       <c r="H5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>18</v>
+      <c r="I5" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>15</v>
@@ -920,30 +832,30 @@
         <v>18</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>17</v>
@@ -952,59 +864,59 @@
         <v>18</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="3" t="s">
-        <v>18</v>
+      <c r="I8" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>16</v>
@@ -1013,30 +925,30 @@
         <v>17</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>16</v>
@@ -1045,330 +957,74 @@
         <v>17</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>15</v>
+        <v>68</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="4" t="s">
-        <v>23</v>
+      <c r="I12" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J14" s="2" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="I20" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated production release with live Owner Admin portal, MongoDB Atlas sync, and responsive modal layout
</commit_message>
<xml_diff>
--- a/data/b2b_bookings.xlsx
+++ b/data/b2b_bookings.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="75">
   <si>
     <t>Booking ID</t>
   </si>
@@ -43,6 +43,36 @@
     <t>Created At (Timestamp)</t>
   </si>
   <si>
+    <t>B2B-8058</t>
+  </si>
+  <si>
+    <t>Hdjjdkd</t>
+  </si>
+  <si>
+    <t>1236458798</t>
+  </si>
+  <si>
+    <t>Bridal &amp; Event Makeover Packages</t>
+  </si>
+  <si>
+    <t>₹7999</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>09:30 AM (Morning)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Confirmed</t>
+  </si>
+  <si>
+    <t>1/10/2026, 6:59:15 pm</t>
+  </si>
+  <si>
     <t>B2B-7652</t>
   </si>
   <si>
@@ -58,18 +88,9 @@
     <t>₹1999</t>
   </si>
   <si>
-    <t>2026-10-01</t>
-  </si>
-  <si>
     <t>11:00 AM (Morning)</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Confirmed</t>
-  </si>
-  <si>
     <t>1/10/2026, 6:21:22 pm</t>
   </si>
   <si>
@@ -77,12 +98,6 @@
   </si>
   <si>
     <t>9632581470</t>
-  </si>
-  <si>
-    <t>Bridal &amp; Event Makeover Packages</t>
-  </si>
-  <si>
-    <t>₹7999</t>
   </si>
   <si>
     <t>1/10/2026, 6:16:45 pm</t>
@@ -628,7 +643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -712,22 +727,22 @@
         <v>20</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>17</v>
@@ -736,30 +751,30 @@
         <v>18</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>17</v>
@@ -768,94 +783,94 @@
         <v>18</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="H5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="3" t="s">
-        <v>18</v>
+      <c r="I6" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>17</v>
@@ -864,68 +879,68 @@
         <v>18</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="G8" s="2" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="4" t="s">
-        <v>36</v>
+      <c r="I8" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>58</v>
@@ -942,89 +957,121 @@
         <v>61</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>15</v>
+        <v>62</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>68</v>
+        <v>15</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="2" t="s">
-        <v>69</v>
+      <c r="J13" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>